<commit_message>
fix: Semiconductor Testing base equipment weights
Computer/Laptop, Printer and Multimedia Projector 8/6/7 -> 5/5/5, the
weight these rows carry across the rest of the standards. Sum 161 -> 155.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/xlsx/bsia--semiconductor-testing-engineering.xlsx
+++ b/data/xlsx/bsia--semiconductor-testing-engineering.xlsx
@@ -655,7 +655,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F16" s="9">
         <f>IFERROR(MIN(C16,D16)*E16/C16,0)</f>
@@ -679,7 +679,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F17" s="9">
         <f>IFERROR(MIN(C17,D17)*E17/C17,0)</f>
@@ -703,7 +703,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F18" s="9">
         <f>IFERROR(MIN(C18,D18)*E18/C18,0)</f>

</xml_diff>

<commit_message>
fix: merge Semiconductor Testing computer rows
Trainer computer and the 25 trainee workstations become one row,
required 26, weight 10, first in the list. 21 items -> 20, sum 155 -> 151.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/xlsx/bsia--semiconductor-testing-engineering.xlsx
+++ b/data/xlsx/bsia--semiconductor-testing-engineering.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
@@ -132,6 +132,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -503,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.17" customWidth="1" min="1" max="1"/>
@@ -640,22 +652,22 @@
       </c>
     </row>
     <row r="16" ht="14.15" customHeight="1">
-      <c r="A16" s="14" t="n">
+      <c r="A16" s="18" t="n">
         <v>1</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Computer/Laptop (Trainer)</t>
+          <t>High-performance Desktop/Laptop Workstation (25 trainees + 01 trainer)</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="D16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F16" s="9">
         <f>IFERROR(MIN(C16,D16)*E16/C16,0)</f>
@@ -664,7 +676,7 @@
       <c r="G16" s="9" t="n"/>
     </row>
     <row r="17" ht="14.15" customHeight="1">
-      <c r="A17" s="14" t="n">
+      <c r="A17" s="18" t="n">
         <v>2</v>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -688,7 +700,7 @@
       <c r="G17" s="9" t="n"/>
     </row>
     <row r="18" ht="14.15" customHeight="1">
-      <c r="A18" s="14" t="n">
+      <c r="A18" s="18" t="n">
         <v>3</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -712,12 +724,12 @@
       <c r="G18" s="9" t="n"/>
     </row>
     <row r="19" ht="14.15" customHeight="1">
-      <c r="A19" s="14" t="n">
+      <c r="A19" s="18" t="n">
         <v>4</v>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>High-performance Desktop/Laptop Workstation</t>
+          <t>ATE Test Program Development Software (Advantest SmarTest Offline/Simulator or equivalent ATE simulation environment)</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
@@ -727,7 +739,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F19" s="9">
         <f>IFERROR(MIN(C19,D19)*E19/C19,0)</f>
@@ -736,12 +748,12 @@
       <c r="G19" s="9" t="n"/>
     </row>
     <row r="20" ht="14.15" customHeight="1">
-      <c r="A20" s="14" t="n">
+      <c r="A20" s="18" t="n">
         <v>5</v>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>ATE Test Program Development Software (Advantest SmarTest Offline/Simulator or equivalent ATE simulation environment)</t>
+          <t>Data Analysis Software (Spreadsheet/Statistical/Scripting Tools)</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
@@ -751,7 +763,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F20" s="9">
         <f>IFERROR(MIN(C20,D20)*E20/C20,0)</f>
@@ -760,12 +772,12 @@
       <c r="G20" s="9" t="n"/>
     </row>
     <row r="21" ht="14.15" customHeight="1">
-      <c r="A21" s="14" t="n">
+      <c r="A21" s="18" t="n">
         <v>6</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Data Analysis Software (Spreadsheet/Statistical/Scripting Tools)</t>
+          <t>Digital Multimeter</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
@@ -775,7 +787,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F21" s="9">
         <f>IFERROR(MIN(C21,D21)*E21/C21,0)</f>
@@ -784,12 +796,12 @@
       <c r="G21" s="9" t="n"/>
     </row>
     <row r="22" ht="14.15" customHeight="1">
-      <c r="A22" s="14" t="n">
+      <c r="A22" s="18" t="n">
         <v>7</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Digital Multimeter</t>
+          <t>ESD-safe Workbench with ESD Mat and Wrist Strap</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
@@ -799,7 +811,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F22" s="9">
         <f>IFERROR(MIN(C22,D22)*E22/C22,0)</f>
@@ -808,12 +820,12 @@
       <c r="G22" s="9" t="n"/>
     </row>
     <row r="23" ht="14.15" customHeight="1">
-      <c r="A23" s="14" t="n">
+      <c r="A23" s="18" t="n">
         <v>8</v>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>ESD-safe Workbench with ESD Mat and Wrist Strap</t>
+          <t>Sample IC Devices and Test Boards (Digital, Analog, Mixed-Signal)</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
@@ -823,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F23" s="9">
         <f>IFERROR(MIN(C23,D23)*E23/C23,0)</f>
@@ -832,12 +844,12 @@
       <c r="G23" s="9" t="n"/>
     </row>
     <row r="24" ht="14.15" customHeight="1">
-      <c r="A24" s="14" t="n">
+      <c r="A24" s="18" t="n">
         <v>9</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Sample IC Devices and Test Boards (Digital, Analog, Mixed-Signal)</t>
+          <t>Breadboard and Electronic Component Kits</t>
         </is>
       </c>
       <c r="C24" s="9" t="n">
@@ -847,7 +859,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F24" s="9">
         <f>IFERROR(MIN(C24,D24)*E24/C24,0)</f>
@@ -856,22 +868,22 @@
       <c r="G24" s="9" t="n"/>
     </row>
     <row r="25" ht="14.15" customHeight="1">
-      <c r="A25" s="14" t="n">
+      <c r="A25" s="18" t="n">
         <v>10</v>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Breadboard and Electronic Component Kits</t>
+          <t>Digital Storage Oscilloscope</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D25" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F25" s="9">
         <f>IFERROR(MIN(C25,D25)*E25/C25,0)</f>
@@ -880,12 +892,12 @@
       <c r="G25" s="9" t="n"/>
     </row>
     <row r="26" ht="14.15" customHeight="1">
-      <c r="A26" s="14" t="n">
+      <c r="A26" s="18" t="n">
         <v>11</v>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Digital Storage Oscilloscope</t>
+          <t>DC Regulated Power Supply</t>
         </is>
       </c>
       <c r="C26" s="9" t="n">
@@ -895,7 +907,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F26" s="9">
         <f>IFERROR(MIN(C26,D26)*E26/C26,0)</f>
@@ -904,12 +916,12 @@
       <c r="G26" s="9" t="n"/>
     </row>
     <row r="27" ht="14.15" customHeight="1">
-      <c r="A27" s="14" t="n">
+      <c r="A27" s="18" t="n">
         <v>12</v>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>DC Regulated Power Supply</t>
+          <t>Function/Signal Generator</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
@@ -928,12 +940,12 @@
       <c r="G27" s="9" t="n"/>
     </row>
     <row r="28" ht="14.15" customHeight="1">
-      <c r="A28" s="14" t="n">
+      <c r="A28" s="18" t="n">
         <v>13</v>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Function/Signal Generator</t>
+          <t>Logic Analyzer</t>
         </is>
       </c>
       <c r="C28" s="9" t="n">
@@ -952,16 +964,16 @@
       <c r="G28" s="9" t="n"/>
     </row>
     <row r="29" ht="14.15" customHeight="1">
-      <c r="A29" s="14" t="n">
+      <c r="A29" s="18" t="n">
         <v>14</v>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Logic Analyzer</t>
+          <t>Sample Loadboard/DUT Board and Socket Demonstration Kits</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D29" s="9" t="n">
         <v>0</v>
@@ -976,22 +988,22 @@
       <c r="G29" s="9" t="n"/>
     </row>
     <row r="30" ht="14.15" customHeight="1">
-      <c r="A30" s="14" t="n">
+      <c r="A30" s="18" t="n">
         <v>15</v>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Sample Loadboard/DUT Board and Socket Demonstration Kits</t>
+          <t>Probe Card and Test Fixture Illustration/Demonstration Set</t>
         </is>
       </c>
       <c r="C30" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" s="9">
         <f>IFERROR(MIN(C30,D30)*E30/C30,0)</f>
@@ -1000,36 +1012,40 @@
       <c r="G30" s="9" t="n"/>
     </row>
     <row r="31" ht="14.15" customHeight="1">
-      <c r="A31" s="14" t="n">
+      <c r="A31" s="18" t="n">
         <v>16</v>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Probe Card and Test Fixture Illustration/Demonstration Set</t>
+          <t>ATE Access or Remote/Partner ATE Facility (Advantest V93000 or equivalent) for Demonstration</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="9" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F31" s="9">
         <f>IFERROR(MIN(C31,D31)*E31/C31,0)</f>
         <v/>
       </c>
-      <c r="G31" s="9" t="n"/>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>01 set</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="14.15" customHeight="1">
-      <c r="A32" s="14" t="n">
+      <c r="A32" s="18" t="n">
         <v>17</v>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>ATE Access or Remote/Partner ATE Facility (Advantest V93000 or equivalent) for Demonstration</t>
+          <t>Sample Production Test Data Sets (STDF/CSV) with Analysis Templates</t>
         </is>
       </c>
       <c r="C32" s="9" t="n">
@@ -1039,7 +1055,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F32" s="9">
         <f>IFERROR(MIN(C32,D32)*E32/C32,0)</f>
@@ -1052,12 +1068,12 @@
       </c>
     </row>
     <row r="33" ht="14.15" customHeight="1">
-      <c r="A33" s="14" t="n">
+      <c r="A33" s="18" t="n">
         <v>18</v>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Sample Production Test Data Sets (STDF/CSV) with Analysis Templates</t>
+          <t>Internet Connectivity with Network Switch and Router</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
@@ -1067,25 +1083,21 @@
         <v>0</v>
       </c>
       <c r="E33" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F33" s="9">
         <f>IFERROR(MIN(C33,D33)*E33/C33,0)</f>
         <v/>
       </c>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>01 set</t>
-        </is>
-      </c>
+      <c r="G33" s="9" t="n"/>
     </row>
     <row r="34" ht="14.15" customHeight="1">
-      <c r="A34" s="14" t="n">
+      <c r="A34" s="18" t="n">
         <v>19</v>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Internet Connectivity with Network Switch and Router</t>
+          <t>Central File/Storage Server</t>
         </is>
       </c>
       <c r="C34" s="9" t="n">
@@ -1104,12 +1116,12 @@
       <c r="G34" s="9" t="n"/>
     </row>
     <row r="35" ht="14.15" customHeight="1">
-      <c r="A35" s="14" t="n">
+      <c r="A35" s="18" t="n">
         <v>20</v>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Central File/Storage Server</t>
+          <t>First Aid and Fire Safety Equipment</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
@@ -1119,93 +1131,69 @@
         <v>0</v>
       </c>
       <c r="E35" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F35" s="9">
         <f>IFERROR(MIN(C35,D35)*E35/C35,0)</f>
         <v/>
       </c>
-      <c r="G35" s="9" t="n"/>
-    </row>
-    <row r="36" ht="14.15" customHeight="1">
-      <c r="A36" s="14" t="n">
-        <v>21</v>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>First Aid and Fire Safety Equipment</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="F36" s="9">
-        <f>IFERROR(MIN(C36,D36)*E36/C36,0)</f>
-        <v/>
-      </c>
-      <c r="G36" s="9" t="inlineStr">
+      <c r="G35" s="9" t="inlineStr">
         <is>
           <t>01 set</t>
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>Sum</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="12" t="n"/>
+      <c r="E36" s="19">
+        <f>SUM(E16:E35)</f>
+        <v/>
+      </c>
+      <c r="F36" s="19">
+        <f>SUM(F16:F35)</f>
+        <v/>
+      </c>
+      <c r="G36" s="13" t="n"/>
+    </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
-        <is>
-          <t>Sum</t>
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>Score out of 100</t>
         </is>
       </c>
       <c r="B37" s="11" t="n"/>
       <c r="C37" s="11" t="n"/>
-      <c r="D37" s="12" t="n"/>
-      <c r="E37" s="15">
-        <f>SUM(E16:E36)</f>
-        <v/>
-      </c>
-      <c r="F37" s="15">
-        <f>SUM(F16:F36)</f>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="19">
+        <f>F36/E36*100</f>
         <v/>
       </c>
       <c r="G37" s="13" t="n"/>
     </row>
-    <row r="38">
-      <c r="A38" s="15" t="inlineStr">
-        <is>
-          <t>Score out of 100</t>
-        </is>
-      </c>
-      <c r="B38" s="11" t="n"/>
-      <c r="C38" s="11" t="n"/>
-      <c r="D38" s="11" t="n"/>
-      <c r="E38" s="12" t="n"/>
-      <c r="F38" s="15">
-        <f>F37/E37*100</f>
-        <v/>
-      </c>
-      <c r="G38" s="13" t="n"/>
-    </row>
-    <row r="39" ht="9.75" customHeight="1"/>
-    <row r="40">
-      <c r="A40" s="15" t="inlineStr">
+    <row r="38" ht="9.75" customHeight="1"/>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">Total achieved points out of 30  </t>
         </is>
       </c>
-      <c r="B40" s="11" t="n"/>
-      <c r="C40" s="11" t="n"/>
-      <c r="D40" s="11" t="n"/>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="15">
-        <f>F38*30/100</f>
-        <v/>
-      </c>
-      <c r="G40" s="15" t="inlineStr">
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="19">
+        <f>F37*30/100</f>
+        <v/>
+      </c>
+      <c r="G39" s="19" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
@@ -1214,13 +1202,13 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A37:E37"/>
     <mergeCell ref="C8:G8"/>
-    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>